<commit_message>
Program now checks for duplicate parts and puts warning on the cutsheet for the different identical part cases
</commit_message>
<xml_diff>
--- a/CutlistTestSheet.xlsx
+++ b/CutlistTestSheet.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\TimAllen\source\repos\timallenyi111\ExcelCutlistGenerator\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D9C3A9F0-9140-4359-8DEB-EA4033E876CB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4A700F7D-C9A9-42F4-B228-C340DFF613B2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="38620" windowHeight="21100" xr2:uid="{A04337D9-4362-4FDA-A529-445F1762424B}"/>
+    <workbookView xWindow="-90" yWindow="0" windowWidth="19380" windowHeight="20970" xr2:uid="{A04337D9-4362-4FDA-A529-445F1762424B}"/>
   </bookViews>
   <sheets>
     <sheet name="Parts" sheetId="1" r:id="rId1"/>
@@ -60,7 +60,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="64" uniqueCount="43">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="75" uniqueCount="44">
   <si>
     <t>Part Number</t>
   </si>
@@ -189,19 +189,28 @@
   </si>
   <si>
     <t>L4x4x1/4</t>
+  </si>
+  <si>
+    <t>HSS3X3X1/8</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="1" x14ac:knownFonts="1">
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Aptos Narrow"/>
       <family val="2"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF000000"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
     </font>
   </fonts>
   <fills count="3">
@@ -657,7 +666,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4AF4D0D2-226A-4E4B-91A1-4F092F814998}">
   <sheetPr codeName="Sheet1"/>
-  <dimension ref="A1:I14"/>
+  <dimension ref="A1:I17"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="14.36328125" customWidth="1"/>
@@ -698,7 +707,7 @@
         <v>5</v>
       </c>
       <c r="I2">
-        <f>B2+B3+B4+B9</f>
+        <f>B2+B3+B4+B10</f>
         <v>239.8125</v>
       </c>
     </row>
@@ -742,10 +751,10 @@
     </row>
     <row r="5" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="B5" t="s">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="C5" s="1" t="s">
         <v>6</v>
@@ -753,16 +762,14 @@
       <c r="D5" s="4" t="s">
         <v>29</v>
       </c>
-      <c r="E5" s="4" t="s">
-        <v>34</v>
-      </c>
+      <c r="E5" s="4"/>
     </row>
     <row r="6" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="B6" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="C6" s="1" t="s">
         <v>6</v>
@@ -771,15 +778,15 @@
         <v>29</v>
       </c>
       <c r="E6" s="4" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
     </row>
     <row r="7" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="B7" t="s">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="C7" s="1" t="s">
         <v>6</v>
@@ -788,15 +795,15 @@
         <v>29</v>
       </c>
       <c r="E7" s="4" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
     </row>
     <row r="8" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A8" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="B8" t="s">
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="C8" s="1" t="s">
         <v>6</v>
@@ -805,49 +812,49 @@
         <v>29</v>
       </c>
       <c r="E8" s="4" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
     </row>
     <row r="9" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A9" t="s">
-        <v>19</v>
+        <v>17</v>
       </c>
       <c r="B9" t="s">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="C9" s="1" t="s">
-        <v>21</v>
+        <v>6</v>
       </c>
       <c r="D9" s="4" t="s">
         <v>29</v>
       </c>
       <c r="E9" s="4" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
     </row>
     <row r="10" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A10" t="s">
-        <v>22</v>
+        <v>19</v>
       </c>
       <c r="B10" t="s">
-        <v>23</v>
+        <v>20</v>
       </c>
       <c r="C10" s="1" t="s">
-        <v>6</v>
+        <v>21</v>
       </c>
       <c r="D10" s="4" t="s">
         <v>29</v>
       </c>
       <c r="E10" s="4" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
     </row>
     <row r="11" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A11" t="s">
-        <v>24</v>
+        <v>22</v>
       </c>
       <c r="B11" t="s">
-        <v>25</v>
+        <v>23</v>
       </c>
       <c r="C11" s="1" t="s">
         <v>6</v>
@@ -856,55 +863,100 @@
         <v>29</v>
       </c>
       <c r="E11" s="4" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
     </row>
     <row r="12" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A12" t="s">
-        <v>26</v>
+        <v>24</v>
       </c>
       <c r="B12" t="s">
-        <v>27</v>
+        <v>25</v>
       </c>
       <c r="C12" s="1" t="s">
-        <v>28</v>
+        <v>6</v>
       </c>
       <c r="D12" s="4" t="s">
         <v>29</v>
       </c>
       <c r="E12" s="4" t="s">
-        <v>27</v>
+        <v>40</v>
       </c>
     </row>
     <row r="13" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A13" t="s">
-        <v>30</v>
-      </c>
-      <c r="B13" s="5">
-        <v>20.6875</v>
-      </c>
-      <c r="C13" s="1">
-        <v>2</v>
+        <v>26</v>
+      </c>
+      <c r="B13" t="s">
+        <v>27</v>
+      </c>
+      <c r="C13" s="1" t="s">
+        <v>28</v>
       </c>
       <c r="D13" s="4" t="s">
-        <v>31</v>
-      </c>
-      <c r="E13">
-        <v>20.6875</v>
+        <v>29</v>
+      </c>
+      <c r="E13" s="4" t="s">
+        <v>27</v>
       </c>
     </row>
     <row r="14" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A14" t="s">
+        <v>30</v>
+      </c>
+      <c r="B14" s="5">
+        <v>20.6875</v>
+      </c>
+      <c r="C14" s="1">
+        <v>2</v>
+      </c>
+      <c r="D14" s="4" t="s">
+        <v>31</v>
+      </c>
+      <c r="E14">
+        <v>20.6875</v>
+      </c>
+    </row>
+    <row r="15" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A15" t="s">
         <v>41</v>
       </c>
-      <c r="B14">
+      <c r="B15">
         <v>32</v>
       </c>
-      <c r="C14" s="1">
+      <c r="C15" s="1">
         <v>10</v>
       </c>
-      <c r="D14" s="4" t="s">
+      <c r="D15" s="4" t="s">
         <v>42</v>
+      </c>
+    </row>
+    <row r="16" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A16" t="s">
+        <v>17</v>
+      </c>
+      <c r="B16">
+        <v>32</v>
+      </c>
+      <c r="C16" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="D16" s="4" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="17" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A17" t="s">
+        <v>24</v>
+      </c>
+      <c r="B17" t="s">
+        <v>25</v>
+      </c>
+      <c r="C17" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="D17" s="4" t="s">
+        <v>43</v>
       </c>
     </row>
   </sheetData>
@@ -958,7 +1010,7 @@
     </row>
     <row r="2" spans="1:2" ht="20.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A2" t="str" cm="1">
-        <f t="array" ref="A2:A4">_xlfn.UNIQUE(_xlfn._xlws.FILTER(Parts!D2:D500,Parts!D2:D500&lt;&gt;""))</f>
+        <f t="array" ref="A2:A5">_xlfn.UNIQUE(_xlfn._xlws.FILTER(Parts!D2:D501,Parts!D2:D501&lt;&gt;""))</f>
         <v>HSS2X2X1/8</v>
       </c>
       <c r="B2">
@@ -981,7 +1033,14 @@
         <v>24</v>
       </c>
     </row>
-    <row r="5" spans="1:2" ht="20.5" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="5" spans="1:2" ht="20.5" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A5" t="str">
+        <v>HSS3X3X1/8</v>
+      </c>
+      <c r="B5">
+        <v>20</v>
+      </c>
+    </row>
     <row r="6" spans="1:2" ht="20.5" customHeight="1" x14ac:dyDescent="0.35"/>
     <row r="7" spans="1:2" ht="20.5" customHeight="1" x14ac:dyDescent="0.35"/>
     <row r="8" spans="1:2" ht="20.5" customHeight="1" x14ac:dyDescent="0.35"/>

</xml_diff>